<commit_message>
docs(testcases): sync v2 template suite files with updated test data
</commit_message>
<xml_diff>
--- a/testcases/Functional_TC_Dolibarr_v2.xlsx
+++ b/testcases/Functional_TC_Dolibarr_v2.xlsx
@@ -129,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -217,22 +217,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -285,7 +274,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -748,9 +736,9 @@
           <t>Document History – To maintain a list of changes being made</t>
         </is>
       </c>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="8" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -809,9 +797,9 @@
           <t>Reference Documents – Clearly mark the document used as an input to create the test case</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
@@ -847,7 +835,7 @@
           <t>Dolibarr ERP &amp; CRM 22.0.4 (hệ thống kiểm thử)</t>
         </is>
       </c>
-      <c r="E13" s="8" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
@@ -865,7 +853,7 @@
           <t>testcases/Dolibarr_TestCases.xlsx (nguồn test case)</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n"/>
+      <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
@@ -883,7 +871,7 @@
           <t>docs/UseCases.md — UC-01 Sales, UC-02 CRM, UC-03 Stock</t>
         </is>
       </c>
-      <c r="E15" s="8" t="n"/>
+      <c r="E15" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -928,6 +916,15 @@
           <t>TEST REQUIREMENTS — Dolibarr ERP &amp; CRM 22.0.4</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
+      <c r="I1" s="10" t="n"/>
+      <c r="J1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -942,27 +939,27 @@
           <t>Project</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n"/>
+      <c r="B3" s="13" t="n"/>
       <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Kiểm thử phần mềm Dolibarr ERP &amp; CRM 22.0.4</t>
         </is>
       </c>
-      <c r="D3" s="24" t="n"/>
-      <c r="E3" s="24" t="n"/>
-      <c r="F3" s="8" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
       <c r="G3" s="12" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="H3" s="8" t="n"/>
+      <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="inlineStr">
         <is>
           <t>CRM · Sales &amp; Invoicing · Stock</t>
         </is>
       </c>
-      <c r="J3" s="8" t="n"/>
+      <c r="J3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -970,27 +967,27 @@
           <t>Test Designed By</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
+      <c r="B4" s="13" t="n"/>
       <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Đặng Hải Phi (23DH112608)</t>
         </is>
       </c>
-      <c r="D4" s="24" t="n"/>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="8" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="13" t="n"/>
       <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Reviewed By</t>
         </is>
       </c>
-      <c r="H4" s="8" t="n"/>
+      <c r="H4" s="13" t="n"/>
       <c r="I4" s="13" t="inlineStr">
         <is>
           <t>Đặng Hải Phi (tự rà soát – đồ án cá nhân)</t>
         </is>
       </c>
-      <c r="J4" s="8" t="n"/>
+      <c r="J4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -998,27 +995,27 @@
           <t>Test Designed Date</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
+      <c r="B5" s="13" t="n"/>
       <c r="C5" s="13" t="inlineStr">
         <is>
           <t>05-Oct-2026</t>
         </is>
       </c>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="8" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
       <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Reviewed Date</t>
         </is>
       </c>
-      <c r="H5" s="8" t="n"/>
+      <c r="H5" s="13" t="n"/>
       <c r="I5" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="8" t="n"/>
+      <c r="J5" s="13" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1026,15 +1023,15 @@
           <t>List of Test Requirements</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n"/>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="24" t="n"/>
-      <c r="I7" s="24" t="n"/>
-      <c r="J7" s="8" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1094,15 +1091,15 @@
           <t>Module CRM — Quản lý khách hàng (UC-02)</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n"/>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="24" t="n"/>
-      <c r="I9" s="24" t="n"/>
-      <c r="J9" s="8" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
     </row>
     <row r="10" ht="195" customHeight="1">
       <c r="A10" s="14" t="n">
@@ -1328,15 +1325,15 @@
           <t>Module Sales &amp; Invoicing — Báo giá &amp; Hóa đơn (UC-01)</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n"/>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="24" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="24" t="n"/>
-      <c r="I14" s="24" t="n"/>
-      <c r="J14" s="8" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
     </row>
     <row r="15" ht="195" customHeight="1">
       <c r="A15" s="14" t="n">
@@ -1519,15 +1516,15 @@
           <t>Module Stock — Quản lý kho (UC-03)</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
-      <c r="I18" s="24" t="n"/>
-      <c r="J18" s="8" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19" ht="46.5" customHeight="1">
       <c r="A19" s="14" t="n">
@@ -1744,6 +1741,22 @@
           <t>TEST CASES — CRM — Quản lý khách hàng (UC-02)</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
+      <c r="I1" s="10" t="n"/>
+      <c r="J1" s="10" t="n"/>
+      <c r="K1" s="10" t="n"/>
+      <c r="L1" s="10" t="n"/>
+      <c r="M1" s="10" t="n"/>
+      <c r="N1" s="10" t="n"/>
+      <c r="O1" s="10" t="n"/>
+      <c r="P1" s="10" t="n"/>
+      <c r="Q1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -1845,22 +1858,22 @@
           <t>Functional TCs</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n"/>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
-      <c r="I5" s="24" t="n"/>
-      <c r="J5" s="24" t="n"/>
-      <c r="K5" s="24" t="n"/>
-      <c r="L5" s="24" t="n"/>
-      <c r="M5" s="24" t="n"/>
-      <c r="N5" s="24" t="n"/>
-      <c r="O5" s="24" t="n"/>
-      <c r="P5" s="24" t="n"/>
-      <c r="Q5" s="8" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1868,22 +1881,22 @@
           <t>F-CRM-01 · Tạo khách hàng mới   (14 test case)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="24" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="8" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="14" t="n">
@@ -3040,7 +3053,7 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống từ chối lưu và hiển thị thông báo lỗi: Đợt 1 ('abc@'): 'Email address abc@ is incorrect'; Đợt 2 ('abc.com'): 'Email address abc.com is incorrect'. URL giữ nguyên card.php, không sinh Third-party mới.</t>
+          <t>Lần 1 (nhập 'abc@'): Error='Email address abc@ is incorrect'. Lần 2 (nhập 'abc.com'): Error='Email address abc.com is incorrect'. Không lưu bản ghi nào.</t>
         </is>
       </c>
       <c r="P35" s="14" t="inlineStr"/>
@@ -3935,22 +3948,22 @@
           <t>F-CRM-02 · Chỉnh sửa thông tin khách hàng   (5 test case)</t>
         </is>
       </c>
-      <c r="B59" s="24" t="n"/>
-      <c r="C59" s="24" t="n"/>
-      <c r="D59" s="24" t="n"/>
-      <c r="E59" s="24" t="n"/>
-      <c r="F59" s="24" t="n"/>
-      <c r="G59" s="24" t="n"/>
-      <c r="H59" s="24" t="n"/>
-      <c r="I59" s="24" t="n"/>
-      <c r="J59" s="24" t="n"/>
-      <c r="K59" s="24" t="n"/>
-      <c r="L59" s="24" t="n"/>
-      <c r="M59" s="24" t="n"/>
-      <c r="N59" s="24" t="n"/>
-      <c r="O59" s="24" t="n"/>
-      <c r="P59" s="24" t="n"/>
-      <c r="Q59" s="8" t="n"/>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="4" t="n"/>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="n"/>
+      <c r="K59" s="4" t="n"/>
+      <c r="L59" s="4" t="n"/>
+      <c r="M59" s="4" t="n"/>
+      <c r="N59" s="4" t="n"/>
+      <c r="O59" s="4" t="n"/>
+      <c r="P59" s="4" t="n"/>
+      <c r="Q59" s="4" t="n"/>
     </row>
     <row r="60" ht="18.5" customHeight="1">
       <c r="A60" s="14" t="n">
@@ -4681,22 +4694,22 @@
           <t>F-CRM-03 · Tìm kiếm khách hàng   (8 test case)</t>
         </is>
       </c>
-      <c r="B80" s="24" t="n"/>
-      <c r="C80" s="24" t="n"/>
-      <c r="D80" s="24" t="n"/>
-      <c r="E80" s="24" t="n"/>
-      <c r="F80" s="24" t="n"/>
-      <c r="G80" s="24" t="n"/>
-      <c r="H80" s="24" t="n"/>
-      <c r="I80" s="24" t="n"/>
-      <c r="J80" s="24" t="n"/>
-      <c r="K80" s="24" t="n"/>
-      <c r="L80" s="24" t="n"/>
-      <c r="M80" s="24" t="n"/>
-      <c r="N80" s="24" t="n"/>
-      <c r="O80" s="24" t="n"/>
-      <c r="P80" s="24" t="n"/>
-      <c r="Q80" s="8" t="n"/>
+      <c r="B80" s="4" t="n"/>
+      <c r="C80" s="4" t="n"/>
+      <c r="D80" s="4" t="n"/>
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="n"/>
+      <c r="K80" s="4" t="n"/>
+      <c r="L80" s="4" t="n"/>
+      <c r="M80" s="4" t="n"/>
+      <c r="N80" s="4" t="n"/>
+      <c r="O80" s="4" t="n"/>
+      <c r="P80" s="4" t="n"/>
+      <c r="Q80" s="4" t="n"/>
     </row>
     <row r="81" ht="32" customHeight="1">
       <c r="A81" s="14" t="n">
@@ -5746,22 +5759,22 @@
           <t>F-CRM-04 · Xóa khách hàng   (5 test case)</t>
         </is>
       </c>
-      <c r="B107" s="24" t="n"/>
-      <c r="C107" s="24" t="n"/>
-      <c r="D107" s="24" t="n"/>
-      <c r="E107" s="24" t="n"/>
-      <c r="F107" s="24" t="n"/>
-      <c r="G107" s="24" t="n"/>
-      <c r="H107" s="24" t="n"/>
-      <c r="I107" s="24" t="n"/>
-      <c r="J107" s="24" t="n"/>
-      <c r="K107" s="24" t="n"/>
-      <c r="L107" s="24" t="n"/>
-      <c r="M107" s="24" t="n"/>
-      <c r="N107" s="24" t="n"/>
-      <c r="O107" s="24" t="n"/>
-      <c r="P107" s="24" t="n"/>
-      <c r="Q107" s="8" t="n"/>
+      <c r="B107" s="4" t="n"/>
+      <c r="C107" s="4" t="n"/>
+      <c r="D107" s="4" t="n"/>
+      <c r="E107" s="4" t="n"/>
+      <c r="F107" s="4" t="n"/>
+      <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
+      <c r="I107" s="4" t="n"/>
+      <c r="J107" s="4" t="n"/>
+      <c r="K107" s="4" t="n"/>
+      <c r="L107" s="4" t="n"/>
+      <c r="M107" s="4" t="n"/>
+      <c r="N107" s="4" t="n"/>
+      <c r="O107" s="4" t="n"/>
+      <c r="P107" s="4" t="n"/>
+      <c r="Q107" s="4" t="n"/>
     </row>
     <row r="108" ht="18.5" customHeight="1">
       <c r="A108" s="14" t="n">
@@ -6455,22 +6468,22 @@
           <t>Look and Feel (GUI) TCs</t>
         </is>
       </c>
-      <c r="B126" s="24" t="n"/>
-      <c r="C126" s="24" t="n"/>
-      <c r="D126" s="24" t="n"/>
-      <c r="E126" s="24" t="n"/>
-      <c r="F126" s="24" t="n"/>
-      <c r="G126" s="24" t="n"/>
-      <c r="H126" s="24" t="n"/>
-      <c r="I126" s="24" t="n"/>
-      <c r="J126" s="24" t="n"/>
-      <c r="K126" s="24" t="n"/>
-      <c r="L126" s="24" t="n"/>
-      <c r="M126" s="24" t="n"/>
-      <c r="N126" s="24" t="n"/>
-      <c r="O126" s="24" t="n"/>
-      <c r="P126" s="24" t="n"/>
-      <c r="Q126" s="8" t="n"/>
+      <c r="B126" s="4" t="n"/>
+      <c r="C126" s="4" t="n"/>
+      <c r="D126" s="4" t="n"/>
+      <c r="E126" s="4" t="n"/>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
+      <c r="I126" s="4" t="n"/>
+      <c r="J126" s="4" t="n"/>
+      <c r="K126" s="4" t="n"/>
+      <c r="L126" s="4" t="n"/>
+      <c r="M126" s="4" t="n"/>
+      <c r="N126" s="4" t="n"/>
+      <c r="O126" s="4" t="n"/>
+      <c r="P126" s="4" t="n"/>
+      <c r="Q126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="18" t="inlineStr">
@@ -6537,9 +6550,9 @@
     <mergeCell ref="J60:J64"/>
     <mergeCell ref="M73:M75"/>
     <mergeCell ref="E98:E100"/>
+    <mergeCell ref="O31:O34"/>
+    <mergeCell ref="C7:C10"/>
     <mergeCell ref="J35:J38"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="O31:O34"/>
     <mergeCell ref="L35:L38"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="O57:O58"/>
@@ -6628,8 +6641,8 @@
     <mergeCell ref="E89:E92"/>
     <mergeCell ref="L96:L97"/>
     <mergeCell ref="B15:B18"/>
+    <mergeCell ref="E76:E79"/>
     <mergeCell ref="O27:O30"/>
-    <mergeCell ref="E76:E79"/>
     <mergeCell ref="D15:D18"/>
     <mergeCell ref="Q27:Q30"/>
     <mergeCell ref="A5:Q5"/>
@@ -6671,9 +6684,9 @@
     <mergeCell ref="O39:O42"/>
     <mergeCell ref="A11:A14"/>
     <mergeCell ref="J46:J48"/>
-    <mergeCell ref="I123:I125"/>
     <mergeCell ref="Q120:Q122"/>
     <mergeCell ref="L46:L48"/>
+    <mergeCell ref="I123:I125"/>
     <mergeCell ref="J15:J18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="L15:L18"/>
@@ -6732,14 +6745,14 @@
     <mergeCell ref="P120:P122"/>
     <mergeCell ref="A46:A48"/>
     <mergeCell ref="K46:K48"/>
+    <mergeCell ref="M46:M48"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="E53:E56"/>
     <mergeCell ref="C46:C48"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="M46:M48"/>
-    <mergeCell ref="E53:E56"/>
-    <mergeCell ref="K15:K18"/>
-    <mergeCell ref="C53:C56"/>
     <mergeCell ref="I15:I18"/>
     <mergeCell ref="E46:E48"/>
+    <mergeCell ref="K15:K18"/>
     <mergeCell ref="N76:N79"/>
     <mergeCell ref="P76:P79"/>
     <mergeCell ref="J101:J103"/>
@@ -7029,6 +7042,22 @@
           <t>TEST CASES — Sales &amp; Invoicing — Báo giá &amp; Hóa đơn (UC-01)</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
+      <c r="I1" s="10" t="n"/>
+      <c r="J1" s="10" t="n"/>
+      <c r="K1" s="10" t="n"/>
+      <c r="L1" s="10" t="n"/>
+      <c r="M1" s="10" t="n"/>
+      <c r="N1" s="10" t="n"/>
+      <c r="O1" s="10" t="n"/>
+      <c r="P1" s="10" t="n"/>
+      <c r="Q1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -7130,22 +7159,22 @@
           <t>Functional TCs</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n"/>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
-      <c r="I5" s="24" t="n"/>
-      <c r="J5" s="24" t="n"/>
-      <c r="K5" s="24" t="n"/>
-      <c r="L5" s="24" t="n"/>
-      <c r="M5" s="24" t="n"/>
-      <c r="N5" s="24" t="n"/>
-      <c r="O5" s="24" t="n"/>
-      <c r="P5" s="24" t="n"/>
-      <c r="Q5" s="8" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -7153,22 +7182,22 @@
           <t>F-SAL-01 · Báo giá thương mại   (8 test case)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="24" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="8" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
     </row>
     <row r="7" ht="18.5" customHeight="1">
       <c r="A7" s="14" t="n">
@@ -8263,22 +8292,22 @@
           <t>F-SAL-02 · Hóa đơn bán hàng chuẩn   (7 test case)</t>
         </is>
       </c>
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="24" t="n"/>
-      <c r="D36" s="24" t="n"/>
-      <c r="E36" s="24" t="n"/>
-      <c r="F36" s="24" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
-      <c r="I36" s="24" t="n"/>
-      <c r="J36" s="24" t="n"/>
-      <c r="K36" s="24" t="n"/>
-      <c r="L36" s="24" t="n"/>
-      <c r="M36" s="24" t="n"/>
-      <c r="N36" s="24" t="n"/>
-      <c r="O36" s="24" t="n"/>
-      <c r="P36" s="24" t="n"/>
-      <c r="Q36" s="8" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
+      <c r="O36" s="4" t="n"/>
+      <c r="P36" s="4" t="n"/>
+      <c r="Q36" s="4" t="n"/>
     </row>
     <row r="37" ht="18.5" customHeight="1">
       <c r="A37" s="14" t="n">
@@ -9231,22 +9260,22 @@
           <t>F-SAL-03 · Hóa đơn đặc biệt   (19 test case)</t>
         </is>
       </c>
-      <c r="B62" s="24" t="n"/>
-      <c r="C62" s="24" t="n"/>
-      <c r="D62" s="24" t="n"/>
-      <c r="E62" s="24" t="n"/>
-      <c r="F62" s="24" t="n"/>
-      <c r="G62" s="24" t="n"/>
-      <c r="H62" s="24" t="n"/>
-      <c r="I62" s="24" t="n"/>
-      <c r="J62" s="24" t="n"/>
-      <c r="K62" s="24" t="n"/>
-      <c r="L62" s="24" t="n"/>
-      <c r="M62" s="24" t="n"/>
-      <c r="N62" s="24" t="n"/>
-      <c r="O62" s="24" t="n"/>
-      <c r="P62" s="24" t="n"/>
-      <c r="Q62" s="8" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n"/>
+      <c r="L62" s="4" t="n"/>
+      <c r="M62" s="4" t="n"/>
+      <c r="N62" s="4" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="n"/>
     </row>
     <row r="63" ht="86" customHeight="1">
       <c r="A63" s="14" t="n">
@@ -10661,7 +10690,7 @@
       </c>
       <c r="O102" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống chặn thanh toán 0.00 € và hiển thị thông báo lỗi 'Field 'Payment amount' is required'. Hóa đơn giữ nguyên trạng thái Not paid, Already paid = 0.00 €.</t>
+          <t>Thông báo lỗi: "Field 'Payment amount' is required". Hóa đơn giữ Not paid; Already paid = 0 €.</t>
         </is>
       </c>
       <c r="P102" s="14" t="inlineStr"/>
@@ -10746,7 +10775,7 @@
       <c r="P105" s="17" t="n"/>
       <c r="Q105" s="17" t="n"/>
     </row>
-    <row r="106" ht="18.5" customHeight="1">
+    <row r="106" ht="45.5" customHeight="1">
       <c r="A106" s="14" t="n">
         <v>25</v>
       </c>
@@ -10791,6 +10820,7 @@
       <c r="J106" s="6" t="inlineStr">
         <is>
           <t>BVA biên dưới âm Amount &lt; 0. Chạy tự động qua Batch2ExtendedTests.
+Flaky: run 20/10 11:06 lỗi timing ở bước chuẩn bị báo giá (độ trễ tải Ajax của Select2 trong CreateAndValidateStandardInvoice(); sản phẩm chưa kịp thêm nên thiếu nút Validate, chờ 10 s). Các lần chạy lại độc lập và lần chạy lại toàn bộ đợt 2 (run 12:49 và 20/10 đơn lẻ) đều Passed.
 Ngày chạy: 2026-10-19</t>
         </is>
       </c>
@@ -10816,7 +10846,7 @@
       </c>
       <c r="O106" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống chặn thanh toán số tiền âm (-50.00 €). Hóa đơn giữ nguyên trạng thái Not paid, Already paid = 0.00 €.</t>
+          <t>Không phát sinh thanh toán âm; hóa đơn giữ Not paid; Already paid = 0 €. Log không ghi nhận thông báo lỗi (Error rỗng).</t>
         </is>
       </c>
       <c r="P106" s="14" t="inlineStr"/>
@@ -10826,7 +10856,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="18.5" customHeight="1">
+    <row r="107" ht="45.5" customHeight="1">
       <c r="A107" s="16" t="n"/>
       <c r="B107" s="16" t="n"/>
       <c r="C107" s="16" t="n"/>
@@ -10851,7 +10881,7 @@
       <c r="P107" s="16" t="n"/>
       <c r="Q107" s="16" t="n"/>
     </row>
-    <row r="108" ht="18.5" customHeight="1">
+    <row r="108" ht="45.5" customHeight="1">
       <c r="A108" s="16" t="n"/>
       <c r="B108" s="16" t="n"/>
       <c r="C108" s="16" t="n"/>
@@ -10876,7 +10906,7 @@
       <c r="P108" s="16" t="n"/>
       <c r="Q108" s="16" t="n"/>
     </row>
-    <row r="109" ht="18.5" customHeight="1">
+    <row r="109" ht="45.5" customHeight="1">
       <c r="A109" s="17" t="n"/>
       <c r="B109" s="17" t="n"/>
       <c r="C109" s="17" t="n"/>
@@ -12055,22 +12085,22 @@
           <t>Look and Feel (GUI) TCs</t>
         </is>
       </c>
-      <c r="B140" s="24" t="n"/>
-      <c r="C140" s="24" t="n"/>
-      <c r="D140" s="24" t="n"/>
-      <c r="E140" s="24" t="n"/>
-      <c r="F140" s="24" t="n"/>
-      <c r="G140" s="24" t="n"/>
-      <c r="H140" s="24" t="n"/>
-      <c r="I140" s="24" t="n"/>
-      <c r="J140" s="24" t="n"/>
-      <c r="K140" s="24" t="n"/>
-      <c r="L140" s="24" t="n"/>
-      <c r="M140" s="24" t="n"/>
-      <c r="N140" s="24" t="n"/>
-      <c r="O140" s="24" t="n"/>
-      <c r="P140" s="24" t="n"/>
-      <c r="Q140" s="8" t="n"/>
+      <c r="B140" s="4" t="n"/>
+      <c r="C140" s="4" t="n"/>
+      <c r="D140" s="4" t="n"/>
+      <c r="E140" s="4" t="n"/>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
+      <c r="I140" s="4" t="n"/>
+      <c r="J140" s="4" t="n"/>
+      <c r="K140" s="4" t="n"/>
+      <c r="L140" s="4" t="n"/>
+      <c r="M140" s="4" t="n"/>
+      <c r="N140" s="4" t="n"/>
+      <c r="O140" s="4" t="n"/>
+      <c r="P140" s="4" t="n"/>
+      <c r="Q140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="18" t="inlineStr">
@@ -12658,6 +12688,22 @@
           <t>TEST CASES — Stock — Quản lý kho (UC-03)</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
+      <c r="I1" s="10" t="n"/>
+      <c r="J1" s="10" t="n"/>
+      <c r="K1" s="10" t="n"/>
+      <c r="L1" s="10" t="n"/>
+      <c r="M1" s="10" t="n"/>
+      <c r="N1" s="10" t="n"/>
+      <c r="O1" s="10" t="n"/>
+      <c r="P1" s="10" t="n"/>
+      <c r="Q1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -12759,22 +12805,22 @@
           <t>Functional TCs</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n"/>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
-      <c r="I5" s="24" t="n"/>
-      <c r="J5" s="24" t="n"/>
-      <c r="K5" s="24" t="n"/>
-      <c r="L5" s="24" t="n"/>
-      <c r="M5" s="24" t="n"/>
-      <c r="N5" s="24" t="n"/>
-      <c r="O5" s="24" t="n"/>
-      <c r="P5" s="24" t="n"/>
-      <c r="Q5" s="8" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -12782,22 +12828,22 @@
           <t>F-STK-02 · Điều chỉnh tồn kho thủ công   (14 test case)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="24" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="8" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="14" t="n">
@@ -14023,7 +14069,7 @@
       <c r="P42" s="17" t="n"/>
       <c r="Q42" s="17" t="n"/>
     </row>
-    <row r="43" ht="32" customHeight="1">
+    <row r="43" ht="18.5" customHeight="1">
       <c r="A43" s="14" t="n">
         <v>8</v>
       </c>
@@ -14093,7 +14139,7 @@
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống chặn và hiển thị lỗi 'Field 'Number of units' is required'. Tồn kho PR002 giữ nguyên 39 → 39, không phát sinh dòng biến động mới trong Stock movements (0 → 0 dòng).</t>
+          <t>Hệ thống báo lỗi "Field 'Number of units' is required". Tồn kho PR002 giữ 39 → 39; số dòng biến động kho 0 → 0.</t>
         </is>
       </c>
       <c r="P43" s="14" t="inlineStr"/>
@@ -14103,7 +14149,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="32" customHeight="1">
+    <row r="44" ht="18.5" customHeight="1">
       <c r="A44" s="16" t="n"/>
       <c r="B44" s="16" t="n"/>
       <c r="C44" s="16" t="n"/>
@@ -14128,7 +14174,7 @@
       <c r="P44" s="16" t="n"/>
       <c r="Q44" s="16" t="n"/>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45" ht="18.5" customHeight="1">
       <c r="A45" s="16" t="n"/>
       <c r="B45" s="16" t="n"/>
       <c r="C45" s="16" t="n"/>
@@ -14153,7 +14199,7 @@
       <c r="P45" s="16" t="n"/>
       <c r="Q45" s="16" t="n"/>
     </row>
-    <row r="46" ht="32" customHeight="1">
+    <row r="46" ht="18.5" customHeight="1">
       <c r="A46" s="17" t="n"/>
       <c r="B46" s="17" t="n"/>
       <c r="C46" s="17" t="n"/>
@@ -14944,22 +14990,22 @@
           <t>F-STK-03 · Cảnh báo tồn kho tối thiểu   (8 test case)</t>
         </is>
       </c>
-      <c r="B67" s="24" t="n"/>
-      <c r="C67" s="24" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="E67" s="24" t="n"/>
-      <c r="F67" s="24" t="n"/>
-      <c r="G67" s="24" t="n"/>
-      <c r="H67" s="24" t="n"/>
-      <c r="I67" s="24" t="n"/>
-      <c r="J67" s="24" t="n"/>
-      <c r="K67" s="24" t="n"/>
-      <c r="L67" s="24" t="n"/>
-      <c r="M67" s="24" t="n"/>
-      <c r="N67" s="24" t="n"/>
-      <c r="O67" s="24" t="n"/>
-      <c r="P67" s="24" t="n"/>
-      <c r="Q67" s="8" t="n"/>
+      <c r="B67" s="4" t="n"/>
+      <c r="C67" s="4" t="n"/>
+      <c r="D67" s="4" t="n"/>
+      <c r="E67" s="4" t="n"/>
+      <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
+      <c r="I67" s="4" t="n"/>
+      <c r="J67" s="4" t="n"/>
+      <c r="K67" s="4" t="n"/>
+      <c r="L67" s="4" t="n"/>
+      <c r="M67" s="4" t="n"/>
+      <c r="N67" s="4" t="n"/>
+      <c r="O67" s="4" t="n"/>
+      <c r="P67" s="4" t="n"/>
+      <c r="Q67" s="4" t="n"/>
     </row>
     <row r="68" ht="45.5" customHeight="1">
       <c r="A68" s="14" t="n">
@@ -15424,7 +15470,7 @@
       <c r="P80" s="17" t="n"/>
       <c r="Q80" s="17" t="n"/>
     </row>
-    <row r="81" ht="32" customHeight="1">
+    <row r="81" ht="59" customHeight="1">
       <c r="A81" s="14" t="n">
         <v>18</v>
       </c>
@@ -15494,7 +15540,7 @@
       </c>
       <c r="O81" s="6" t="inlineStr">
         <is>
-          <t>Chưa thực hiện do thiếu điều kiện tiên quyết tự nhiên (trang Replenishment chỉ có 0/3 sản phẩm dưới ngưỡng cảnh báo). Không can thiệp sửa baseline bằng SQL.</t>
+          <t>Chưa nghiệm thu (Inconclusive, Skipped): trang Replenishment tải trong khoảng 187–918 ms qua các lần chạy (918 ms có log docs/run_dot2_final_20261019_1326.log; 752 ms và 608 ms từ kết quả chạy lại; 187 ms từ lần chạy đầu chưa có log đối chiếu). Số sản phẩm dưới ngưỡng hiển thị 0/3 (thiếu precondition).</t>
         </is>
       </c>
       <c r="P81" s="14" t="inlineStr"/>
@@ -15504,7 +15550,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="32" customHeight="1">
+    <row r="82" ht="59" customHeight="1">
       <c r="A82" s="17" t="n"/>
       <c r="B82" s="17" t="n"/>
       <c r="C82" s="17" t="n"/>
@@ -16003,22 +16049,22 @@
           <t>Look and Feel (GUI) TCs</t>
         </is>
       </c>
-      <c r="B95" s="24" t="n"/>
-      <c r="C95" s="24" t="n"/>
-      <c r="D95" s="24" t="n"/>
-      <c r="E95" s="24" t="n"/>
-      <c r="F95" s="24" t="n"/>
-      <c r="G95" s="24" t="n"/>
-      <c r="H95" s="24" t="n"/>
-      <c r="I95" s="24" t="n"/>
-      <c r="J95" s="24" t="n"/>
-      <c r="K95" s="24" t="n"/>
-      <c r="L95" s="24" t="n"/>
-      <c r="M95" s="24" t="n"/>
-      <c r="N95" s="24" t="n"/>
-      <c r="O95" s="24" t="n"/>
-      <c r="P95" s="24" t="n"/>
-      <c r="Q95" s="8" t="n"/>
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="4" t="n"/>
+      <c r="J95" s="4" t="n"/>
+      <c r="K95" s="4" t="n"/>
+      <c r="L95" s="4" t="n"/>
+      <c r="M95" s="4" t="n"/>
+      <c r="N95" s="4" t="n"/>
+      <c r="O95" s="4" t="n"/>
+      <c r="P95" s="4" t="n"/>
+      <c r="Q95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
@@ -16416,6 +16462,13 @@
           <t>CHECKLIST GUI — Dolibarr ERP &amp; CRM 22.0.4</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -16830,6 +16883,8 @@
           <t>LEGEND — Chú thích</t>
         </is>
       </c>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="11" t="inlineStr">

</xml_diff>